<commit_message>
hide propensity when won
</commit_message>
<xml_diff>
--- a/data/Test.xlsx
+++ b/data/Test.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -510,6 +510,43 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>testt</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Year +1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;br&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>